<commit_message>
Docs: ERS-01 v1.2, CU-01 v2.3 e historias HU-15 a HU-17 con las APIs propias - Camila Olivares
Se agregan los requisitos y casos de uso de las APIs propias, las historias HU-15 a HU-17 con sus criterios (la HU-17 como propuesta) y las tareas S3-13 a S3-18 en el Product Backlog y el Sprint 3. Se cargan las horas reales del sprint, se actualizan los índices y se quitan los RUT del documento de historias.
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/2. Metodología Scrum/SITRAFO_Historias_de_Usuario.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/2. Metodología Scrum/SITRAFO_Historias_de_Usuario.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B1:J24"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.4453125" defaultRowHeight="14.25" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="1.44" customWidth="1" style="12" min="1" max="1"/>
@@ -1026,41 +1026,483 @@
       <c r="I20" s="25" t="n"/>
       <c r="J20" s="25" t="n"/>
     </row>
-    <row r="22" ht="14.25" customHeight="1" s="13">
-      <c r="B22" s="12" t="inlineStr">
+    <row r="21" ht="75" customHeight="1" s="13">
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>E4-H3</t>
+        </is>
+      </c>
+      <c r="C21" s="19" t="inlineStr">
+        <is>
+          <t>Como un cliente</t>
+        </is>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>Necesito consultar el estado de mi pedido con el número de la orden de compra y un código de seguimiento, sin iniciar sesión</t>
+        </is>
+      </c>
+      <c r="E21" s="19" t="inlineStr">
+        <is>
+          <t>Con la finalidad de saber en qué etapa está la fabricación y cuándo lo recibiré, sin tener que llamar a la empresa</t>
+        </is>
+      </c>
+      <c r="F21" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="19" t="inlineStr">
+        <is>
+          <t>Consulta con datos correctos</t>
+        </is>
+      </c>
+      <c r="H21" s="19" t="inlineStr">
+        <is>
+          <t>En caso que el cliente ingrese el número de su orden de compra y el código de seguimiento correcto</t>
+        </is>
+      </c>
+      <c r="I21" s="19" t="inlineStr">
+        <is>
+          <t>cuando presione «Consultar»</t>
+        </is>
+      </c>
+      <c r="J21" s="19" t="inlineStr">
+        <is>
+          <t>el sistema mostrará la etapa actual, el porcentaje de avance, la fecha estimada de entrega y el historial del pedido, sin montos ni datos del cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="75" customHeight="1" s="13">
+      <c r="B22" s="21" t="n"/>
+      <c r="C22" s="21" t="n"/>
+      <c r="D22" s="21" t="n"/>
+      <c r="E22" s="21" t="n"/>
+      <c r="F22" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G22" s="19" t="inlineStr">
+        <is>
+          <t>Código incorrecto o pedido inexistente</t>
+        </is>
+      </c>
+      <c r="H22" s="19" t="inlineStr">
+        <is>
+          <t>En caso que el número no exista o el código no corresponda a la orden</t>
+        </is>
+      </c>
+      <c r="I22" s="19" t="inlineStr">
+        <is>
+          <t>cuando presione «Consultar»</t>
+        </is>
+      </c>
+      <c r="J22" s="19" t="inlineStr">
+        <is>
+          <t>el sistema mostrará el mismo mensaje en ambos casos, «No existe un pedido con ese número y código de seguimiento», sin revelar si el pedido existe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="75" customHeight="1" s="13">
+      <c r="B23" s="21" t="n"/>
+      <c r="C23" s="21" t="n"/>
+      <c r="D23" s="21" t="n"/>
+      <c r="E23" s="21" t="n"/>
+      <c r="F23" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="19" t="inlineStr">
+        <is>
+          <t>Consumidor sin clave de API</t>
+        </is>
+      </c>
+      <c r="H23" s="19" t="inlineStr">
+        <is>
+          <t>En caso que un sistema externo llame a la API sin clave o con una clave inválida</t>
+        </is>
+      </c>
+      <c r="I23" s="19" t="inlineStr">
+        <is>
+          <t>cuando envíe la consulta</t>
+        </is>
+      </c>
+      <c r="J23" s="19" t="inlineStr">
+        <is>
+          <t>el sistema responderá 401 y registrará el intento en el log de integraciones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="75" customHeight="1" s="13">
+      <c r="B24" s="22" t="n"/>
+      <c r="C24" s="22" t="n"/>
+      <c r="D24" s="22" t="n"/>
+      <c r="E24" s="22" t="n"/>
+      <c r="F24" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="G24" s="19" t="inlineStr">
+        <is>
+          <t>Exceso de consultas</t>
+        </is>
+      </c>
+      <c r="H24" s="19" t="inlineStr">
+        <is>
+          <t>En caso que una misma clave supere las 60 consultas en un minuto</t>
+        </is>
+      </c>
+      <c r="I24" s="19" t="inlineStr">
+        <is>
+          <t>cuando envíe una nueva consulta</t>
+        </is>
+      </c>
+      <c r="J24" s="19" t="inlineStr">
+        <is>
+          <t>el sistema responderá 429 hasta que se libere el cupo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="14.25" customHeight="1" s="13">
+      <c r="B25" s="25" t="n"/>
+      <c r="C25" s="25" t="n"/>
+      <c r="D25" s="25" t="n"/>
+      <c r="E25" s="25" t="n"/>
+      <c r="F25" s="24" t="n"/>
+      <c r="G25" s="25" t="n"/>
+      <c r="H25" s="25" t="n"/>
+      <c r="I25" s="25" t="n"/>
+      <c r="J25" s="25" t="n"/>
+    </row>
+    <row r="26" ht="75" customHeight="1" s="13">
+      <c r="B26" s="19" t="inlineStr">
+        <is>
+          <t>E2-H4</t>
+        </is>
+      </c>
+      <c r="C26" s="19" t="inlineStr">
+        <is>
+          <t>Como un cliente o distribuidor</t>
+        </is>
+      </c>
+      <c r="D26" s="19" t="inlineStr">
+        <is>
+          <t>Necesito obtener un precio referencial de uno o más modelos con su cantidad</t>
+        </is>
+      </c>
+      <c r="E26" s="19" t="inlineStr">
+        <is>
+          <t>Con la finalidad de evaluar el costo y el plazo de entrega antes de pedir una cotización formal</t>
+        </is>
+      </c>
+      <c r="F26" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" s="19" t="inlineStr">
+        <is>
+          <t>Estimación correcta</t>
+        </is>
+      </c>
+      <c r="H26" s="19" t="inlineStr">
+        <is>
+          <t>En caso que el modelo esté publicado y la cantidad esté dentro del tope permitido</t>
+        </is>
+      </c>
+      <c r="I26" s="19" t="inlineStr">
+        <is>
+          <t>cuando presione «Estimar»</t>
+        </is>
+      </c>
+      <c r="J26" s="19" t="inlineStr">
+        <is>
+          <t>el sistema mostrará el precio unitario y el total en UF, pesos y dólares, la fecha estimada de entrega y la validez, calculados con el mismo costeo de las cotizaciones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="75" customHeight="1" s="13">
+      <c r="B27" s="21" t="n"/>
+      <c r="C27" s="21" t="n"/>
+      <c r="D27" s="21" t="n"/>
+      <c r="E27" s="21" t="n"/>
+      <c r="F27" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" s="19" t="inlineStr">
+        <is>
+          <t>Sin exponer costos internos</t>
+        </is>
+      </c>
+      <c r="H27" s="19" t="inlineStr">
+        <is>
+          <t>En caso que se consulte cualquier modelo</t>
+        </is>
+      </c>
+      <c r="I27" s="19" t="inlineStr">
+        <is>
+          <t>cuando el sistema responda la estimación</t>
+        </is>
+      </c>
+      <c r="J27" s="19" t="inlineStr">
+        <is>
+          <t>la respuesta no incluirá costos de materiales, horas hombre, recargos ni margen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="75" customHeight="1" s="13">
+      <c r="B28" s="21" t="n"/>
+      <c r="C28" s="21" t="n"/>
+      <c r="D28" s="21" t="n"/>
+      <c r="E28" s="21" t="n"/>
+      <c r="F28" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="G28" s="19" t="inlineStr">
+        <is>
+          <t>Entrada inválida</t>
+        </is>
+      </c>
+      <c r="H28" s="19" t="inlineStr">
+        <is>
+          <t>En caso que el modelo no exista o no esté publicado, la cantidad esté fuera de rango o se envíen más de 10 modelos</t>
+        </is>
+      </c>
+      <c r="I28" s="19" t="inlineStr">
+        <is>
+          <t>cuando envíe la estimación</t>
+        </is>
+      </c>
+      <c r="J28" s="19" t="inlineStr">
+        <is>
+          <t>el sistema responderá 400 indicando el campo que falla.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="75" customHeight="1" s="13">
+      <c r="B29" s="22" t="n"/>
+      <c r="C29" s="22" t="n"/>
+      <c r="D29" s="22" t="n"/>
+      <c r="E29" s="22" t="n"/>
+      <c r="F29" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="G29" s="19" t="inlineStr">
+        <is>
+          <t>Clave sin el servicio</t>
+        </is>
+      </c>
+      <c r="H29" s="19" t="inlineStr">
+        <is>
+          <t>En caso que se use la clave pública del seguimiento, que no tiene el servicio de cotizador</t>
+        </is>
+      </c>
+      <c r="I29" s="19" t="inlineStr">
+        <is>
+          <t>cuando envíe la estimación</t>
+        </is>
+      </c>
+      <c r="J29" s="19" t="inlineStr">
+        <is>
+          <t>el sistema responderá 403 y no entregará precios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="14.25" customHeight="1" s="13">
+      <c r="B30" s="25" t="n"/>
+      <c r="C30" s="25" t="n"/>
+      <c r="D30" s="25" t="n"/>
+      <c r="E30" s="25" t="n"/>
+      <c r="F30" s="24" t="n"/>
+      <c r="G30" s="25" t="n"/>
+      <c r="H30" s="25" t="n"/>
+      <c r="I30" s="25" t="n"/>
+      <c r="J30" s="25" t="n"/>
+    </row>
+    <row r="31" ht="75" customHeight="1" s="13">
+      <c r="B31" s="19" t="inlineStr">
+        <is>
+          <t>E6-H2</t>
+        </is>
+      </c>
+      <c r="C31" s="19" t="inlineStr">
+        <is>
+          <t>Como un proveedor autorizado</t>
+        </is>
+      </c>
+      <c r="D31" s="19" t="inlineStr">
+        <is>
+          <t>Necesito consultar los materiales que están bajo su stock mínimo y la cantidad sugerida de reposición</t>
+        </is>
+      </c>
+      <c r="E31" s="19" t="inlineStr">
+        <is>
+          <t>Con la finalidad de preparar los despachos antes de que la planta se quede sin material</t>
+        </is>
+      </c>
+      <c r="F31" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="19" t="inlineStr">
+        <is>
+          <t>Materiales bajo el mínimo</t>
+        </is>
+      </c>
+      <c r="H31" s="19" t="inlineStr">
+        <is>
+          <t>En caso que uno o más materiales tengan un stock actual inferior a su stock mínimo</t>
+        </is>
+      </c>
+      <c r="I31" s="19" t="inlineStr">
+        <is>
+          <t>cuando el proveedor consulte la API con su clave</t>
+        </is>
+      </c>
+      <c r="J31" s="19" t="inlineStr">
+        <is>
+          <t>el sistema devolverá cada material con su código, nombre, unidad, stock mínimo y cantidad sugerida de reposición, calculados desde el kardex.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="75" customHeight="1" s="13">
+      <c r="B32" s="21" t="n"/>
+      <c r="C32" s="21" t="n"/>
+      <c r="D32" s="21" t="n"/>
+      <c r="E32" s="21" t="n"/>
+      <c r="F32" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G32" s="19" t="inlineStr">
+        <is>
+          <t>Sin materiales bajo el mínimo</t>
+        </is>
+      </c>
+      <c r="H32" s="19" t="inlineStr">
+        <is>
+          <t>En caso que todos los materiales estén sobre su stock mínimo</t>
+        </is>
+      </c>
+      <c r="I32" s="19" t="inlineStr">
+        <is>
+          <t>cuando el proveedor consulte la API</t>
+        </is>
+      </c>
+      <c r="J32" s="19" t="inlineStr">
+        <is>
+          <t>el sistema devolverá una lista vacía junto con la fecha y hora del cálculo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="75" customHeight="1" s="13">
+      <c r="B33" s="21" t="n"/>
+      <c r="C33" s="21" t="n"/>
+      <c r="D33" s="21" t="n"/>
+      <c r="E33" s="21" t="n"/>
+      <c r="F33" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="G33" s="19" t="inlineStr">
+        <is>
+          <t>Clave sin el servicio</t>
+        </is>
+      </c>
+      <c r="H33" s="19" t="inlineStr">
+        <is>
+          <t>En caso que la clave no tenga el servicio de disponibilidad, como la del portal web</t>
+        </is>
+      </c>
+      <c r="I33" s="19" t="inlineStr">
+        <is>
+          <t>cuando consulte la API</t>
+        </is>
+      </c>
+      <c r="J33" s="19" t="inlineStr">
+        <is>
+          <t>el sistema responderá 403 sin entregar información de inventario.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="75" customHeight="1" s="13">
+      <c r="B34" s="22" t="n"/>
+      <c r="C34" s="22" t="n"/>
+      <c r="D34" s="22" t="n"/>
+      <c r="E34" s="22" t="n"/>
+      <c r="F34" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="G34" s="19" t="inlineStr">
+        <is>
+          <t>Consulta registrada</t>
+        </is>
+      </c>
+      <c r="H34" s="19" t="inlineStr">
+        <is>
+          <t>En caso que la consulta sea aceptada o rechazada</t>
+        </is>
+      </c>
+      <c r="I34" s="19" t="inlineStr">
+        <is>
+          <t>cuando el sistema responda</t>
+        </is>
+      </c>
+      <c r="J34" s="19" t="inlineStr">
+        <is>
+          <t>la consulta quedará en el log de integraciones con el consumidor, el resultado y la latencia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="14.25" customHeight="1" s="13">
+      <c r="B35" s="25" t="n"/>
+      <c r="C35" s="25" t="n"/>
+      <c r="D35" s="25" t="n"/>
+      <c r="E35" s="25" t="n"/>
+      <c r="F35" s="24" t="n"/>
+      <c r="G35" s="25" t="n"/>
+      <c r="H35" s="25" t="n"/>
+      <c r="I35" s="25" t="n"/>
+      <c r="J35" s="25" t="n"/>
+    </row>
+    <row r="36"/>
+    <row r="37">
+      <c r="B37" s="12" t="inlineStr">
         <is>
           <t>Nota:</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="14.25" customHeight="1" s="13">
-      <c r="B23" s="12" t="inlineStr">
+    <row r="38">
+      <c r="B38" s="12" t="inlineStr">
         <is>
           <t>- Reemplazar las etiquetas [Rol], [Descripción de la funcionalidad], [Descripción de razón o resultado] por el contenido del enunciado de la historia.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="14.25" customHeight="1" s="13">
-      <c r="B24" s="12" t="inlineStr">
+    <row r="39">
+      <c r="B39" s="12" t="inlineStr">
         <is>
           <t>- Reemplazar las etiquetas [Título del escenario], [contexto], [evento] y [resultado / comportamiento]  por el contenido de los criterios de aceptación.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="C4:F4"/>
+  <mergeCells count="26">
+    <mergeCell ref="B31:B34"/>
+    <mergeCell ref="D31:D34"/>
     <mergeCell ref="G4:J4"/>
+    <mergeCell ref="D6:D9"/>
+    <mergeCell ref="C26:C29"/>
+    <mergeCell ref="B21:B24"/>
+    <mergeCell ref="D21:D24"/>
+    <mergeCell ref="B11:B14"/>
+    <mergeCell ref="D11:D14"/>
+    <mergeCell ref="E31:E34"/>
     <mergeCell ref="C16:C19"/>
-    <mergeCell ref="D6:D9"/>
-    <mergeCell ref="B6:B9"/>
     <mergeCell ref="D16:D19"/>
     <mergeCell ref="E6:E9"/>
+    <mergeCell ref="C21:C24"/>
+    <mergeCell ref="C31:C34"/>
+    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="B6:B9"/>
     <mergeCell ref="C11:C14"/>
     <mergeCell ref="E16:E19"/>
     <mergeCell ref="E11:E14"/>
-    <mergeCell ref="B11:B14"/>
-    <mergeCell ref="D11:D14"/>
+    <mergeCell ref="E26:E29"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="D26:D29"/>
+    <mergeCell ref="E21:E24"/>
     <mergeCell ref="B16:B19"/>
     <mergeCell ref="C6:C9"/>
   </mergeCells>

</xml_diff>